<commit_message>
RMD script is running
</commit_message>
<xml_diff>
--- a/working/CrizerPFAS/CrizerChemIDs.xlsx
+++ b/working/CrizerPFAS/CrizerChemIDs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jwambaug\git\invitrotkstats\working\CrizerPFAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C459F8E6-C802-4346-971A-C157A6A74240}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8032B778-033A-429D-A480-B322183BC9EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{819F4BB0-2119-468F-947F-0171544AB1A3}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{819F4BB0-2119-468F-947F-0171544AB1A3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="159">
   <si>
     <t>Chemical</t>
   </si>
@@ -116,9 +116,6 @@
     <t>DTXSID3031864</t>
   </si>
   <si>
-    <t>Potassium_perfluorobutanesulfonate</t>
-  </si>
-  <si>
     <t>DTXSID3037707</t>
   </si>
   <si>
@@ -354,13 +351,175 @@
   </si>
   <si>
     <t>Perfluoroheptanoyl chloride</t>
+  </si>
+  <si>
+    <t>11-H-Perfluoroundecanoic acid (11H-PFUnDA)</t>
+  </si>
+  <si>
+    <t>6:2 Fluorotelomer sulfonic acid (6:2 FTS)</t>
+  </si>
+  <si>
+    <t>8:2 Fluorotelomer sulfonic acid (8:2 FTS)</t>
+  </si>
+  <si>
+    <t>3:3 Fluorotelomer carboxylic acid (3:3 FTCA)</t>
+  </si>
+  <si>
+    <t>4,4-bis(Trifluoromethyl)-4-fluoropropanoic acid</t>
+  </si>
+  <si>
+    <t>DTXSID80380256</t>
+  </si>
+  <si>
+    <t>6:3 Fluorotelomer carboxylic acid (6:3 FTCA)</t>
+  </si>
+  <si>
+    <t>Perfluoroundecanoic acid (PFUnDA)</t>
+  </si>
+  <si>
+    <t>Perfluoro-3,6-dioxadecanoic acid (PFPE-5)</t>
+  </si>
+  <si>
+    <t>DTXSID50381073</t>
+  </si>
+  <si>
+    <t>Perfluorohexanesulfonamide (PFHxSA)</t>
+  </si>
+  <si>
+    <t>Potassium perfluorobutanesulfonate (KPFBS)</t>
+  </si>
+  <si>
+    <t>Potassium perfluorohexanesulfonate (KPFHxS)</t>
+  </si>
+  <si>
+    <t>N-Ethylperfluorooctanesulfonamide (NEtFOSA)</t>
+  </si>
+  <si>
+    <t>Perfluorooctanesulfonamide (PFOSA)</t>
+  </si>
+  <si>
+    <t>DTXSID3038939</t>
+  </si>
+  <si>
+    <t>Sodium perfluorooctanoate (NaPFOA)</t>
+  </si>
+  <si>
+    <t>2H,2H,3H,3H-Perfluorooctanoic acid (5:3 FTCA)</t>
+  </si>
+  <si>
+    <t>3-(Perfluoroisopropyl)-2-propenoic acid</t>
+  </si>
+  <si>
+    <t>3,3-Bis(trifluoromethyl)-2-propenoic acid</t>
+  </si>
+  <si>
+    <t>Potassium perfluorooctanoate (KPFOA)</t>
+  </si>
+  <si>
+    <t>Perfluorodecanoic acid (PFDA)</t>
+  </si>
+  <si>
+    <t>Perfluorotetradecanoic acid (PFTeDA)</t>
+  </si>
+  <si>
+    <t>4:2 Fluorotelomer sulfonic acid (4:2 FTS)</t>
+  </si>
+  <si>
+    <t>Perfluorotridecanoic acid (PFTrDA)</t>
+  </si>
+  <si>
+    <t>Perfluorobutanoic acid (PFBA)</t>
+  </si>
+  <si>
+    <t>Perfluoropropanoic acid (PFPrA)</t>
+  </si>
+  <si>
+    <t>Perfluorononanoic acid (PFNA)</t>
+  </si>
+  <si>
+    <t>Perfluoropentanoic acid (PFPeA)</t>
+  </si>
+  <si>
+    <t>Perfluorooctanoic acid (PFOA)</t>
+  </si>
+  <si>
+    <t>Perfluorohexanoic acid (PFHxA)</t>
+  </si>
+  <si>
+    <t>Ammonium perfluorooctanoate (NH4PFOA)</t>
+  </si>
+  <si>
+    <t>Perfluoroheptanoic acid (PFHpA)</t>
+  </si>
+  <si>
+    <t>Pentadecafluorooctanoyl chloride (PFOA-Cl)</t>
+  </si>
+  <si>
+    <t>Perfluoroheptanoyl chloride (PFHpA-Cl)</t>
+  </si>
+  <si>
+    <t>Perfluoro-3,6-dioxaheptanoic acid (PFPE-3)</t>
+  </si>
+  <si>
+    <t>Perfluoro-3-methoxypropanoic acid (PFPE-2)</t>
+  </si>
+  <si>
+    <t>Perfluoro(4-methoxybutanoic) acid (PFPE-7)</t>
+  </si>
+  <si>
+    <t>Perfluoro-4-isopropoxybutanoic acid (PFPE-1)</t>
+  </si>
+  <si>
+    <t>Perfluoro(2-ethoxyethane)sulfonic acid (PFEOES)</t>
+  </si>
+  <si>
+    <t>Perfluorooctanesulfonamido ammonium iodide</t>
+  </si>
+  <si>
+    <t>Perfluorooctanesulfonate (PFOS-)</t>
+  </si>
+  <si>
+    <t>Perfluoroheptanesulfonic acid (PFHpS)</t>
+  </si>
+  <si>
+    <t>Perfluorooctanesulfonic acid (PFOS)</t>
+  </si>
+  <si>
+    <t>Perfluorohexanesulfonic acid (PFHxS)</t>
+  </si>
+  <si>
+    <t>2,2,2-Trifluoroethyl perfluorobutanesulfonate</t>
+  </si>
+  <si>
+    <t>Sodium perfluorodecanesulfonate (NaPFDS)</t>
+  </si>
+  <si>
+    <t>Potassium perfluorooctanesulfonate (KPFOS)</t>
+  </si>
+  <si>
+    <t>Perfluorobutanesulfonic acid (PFBS)</t>
+  </si>
+  <si>
+    <t>Perfluoro-1-octanesulfonyl chloride (PFOS-Cl)</t>
+  </si>
+  <si>
+    <t>8H-Perfluorooctanoic acid (8H-PFOA)</t>
+  </si>
+  <si>
+    <t>4H-Perfluorobutanoic acid (4H-PFBA)</t>
+  </si>
+  <si>
+    <t>2-(Perfluorohexyl)ethylphosphonic acid</t>
+  </si>
+  <si>
+    <t>N-Methylperfluorooctanesulfonamide (NMeFOSA)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -395,6 +554,11 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -404,7 +568,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -412,12 +576,70 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -434,9 +656,60 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{5E1F694C-8678-4373-9956-EDB95FB920EB}"/>
     <cellStyle name="Normal 2 2" xfId="1" xr:uid="{1EE674AA-962C-4328-8568-01F827C01B4E}"/>
   </cellStyles>
   <dxfs count="3">
@@ -504,8 +777,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61DDEC30-F9B7-48F5-A8B3-DBABB6D1E149}" name="Table1" displayName="Table1" ref="A1:B55" totalsRowShown="0" dataDxfId="2">
-  <autoFilter ref="A1:B55" xr:uid="{61DDEC30-F9B7-48F5-A8B3-DBABB6D1E149}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{61DDEC30-F9B7-48F5-A8B3-DBABB6D1E149}" name="Table1" displayName="Table1" ref="A1:B106" totalsRowShown="0" dataDxfId="2">
+  <autoFilter ref="A1:B106" xr:uid="{61DDEC30-F9B7-48F5-A8B3-DBABB6D1E149}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B106">
+    <sortCondition ref="A1:A106"/>
+  </sortState>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{CF27F945-8CE4-4AC2-B5C3-1FDA67ACBD79}" name="Chemical" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{7AA6CD87-74DC-4D34-B235-20B5844CCA97}" name="DTXSID" dataDxfId="0"/>
@@ -811,10 +1087,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDE8F23D-687E-440F-B10F-6183CD66E1B7}">
-  <dimension ref="A1:B55"/>
+  <dimension ref="A1:B106"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="42.26953125" customWidth="1"/>
     <col min="2" max="2" width="14.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -827,375 +1103,375 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
+      <c r="A2" s="14" t="s">
+        <v>105</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>45</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>5</v>
+        <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
+        <v>157</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
+        <v>150</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>13</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>15</v>
+        <v>122</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>16</v>
+      <c r="A9" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>19</v>
+        <v>123</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>23</v>
+        <v>124</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>108</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>29</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>31</v>
+        <v>87</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>33</v>
+        <v>87</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
-        <v>34</v>
+        <v>109</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>35</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>37</v>
+        <v>128</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>156</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B23" s="2" t="s">
-        <v>45</v>
+        <v>106</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>47</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>49</v>
+      <c r="A25" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" s="1" t="s">
-        <v>50</v>
+        <v>111</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B27" s="2" t="s">
-        <v>53</v>
+        <v>107</v>
+      </c>
+      <c r="B27" s="19" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" s="1" t="s">
-        <v>54</v>
+        <v>4</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>55</v>
+        <v>5</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" s="1" t="s">
-        <v>56</v>
+      <c r="A29" s="5" t="s">
+        <v>101</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>57</v>
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>59</v>
+      <c r="A30" s="16" t="s">
+        <v>155</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>61</v>
+      <c r="A31" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" s="1" t="s">
-        <v>62</v>
+        <v>136</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" s="1" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>67</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="B35" s="2" t="s">
-        <v>69</v>
+        <v>10</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B36" s="2" t="s">
-        <v>71</v>
+      <c r="A36" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>73</v>
+        <v>15</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>75</v>
+        <v>158</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
-        <v>76</v>
+      <c r="A39" s="5" t="s">
+        <v>102</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>79</v>
+      <c r="A40" s="16" t="s">
+        <v>138</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>81</v>
+        <v>89</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>83</v>
+        <v>144</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>85</v>
+        <v>142</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>87</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>91</v>
+      <c r="A45" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>92</v>
+      <c r="A46" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="16" t="s">
         <v>103</v>
       </c>
       <c r="B48" s="2" t="s">
@@ -1203,59 +1479,467 @@
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B49" s="2" t="s">
-        <v>98</v>
+      <c r="A49" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B49" s="19" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A50" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B50" s="2" t="s">
-        <v>99</v>
+      <c r="A50" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="B50" s="19" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>93</v>
+        <v>29</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>11</v>
+        <v>141</v>
+      </c>
+      <c r="B52" s="19" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>94</v>
+        <v>61</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>95</v>
+        <v>143</v>
+      </c>
+      <c r="B54" s="19" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A56" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="B56" s="19" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A57" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B57" s="12" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A58" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A59" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B59" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A60" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A61" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B61" s="12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A62" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B62" s="11" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A63" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" s="12" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A64" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A65" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B65" s="12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A66" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A67" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="B67" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A68" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B68" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A69" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B69" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A70" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A71" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B71" s="12" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A72" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A73" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B73" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A74" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="B74" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A75" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B75" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A76" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="B76" s="20" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A77" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B77" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A78" s="7" t="s">
+        <v>145</v>
+      </c>
+      <c r="B78" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A79" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B79" s="12" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A80" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B80" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A81" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B81" s="12" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A82" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B82" s="11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A83" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B83" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A84" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="B84" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A85" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B85" s="12" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A86" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B86" s="11" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A87" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B87" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A88" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="B88" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A89" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="B89" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A90" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="B90" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A91" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="B91" s="12" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A92" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="B92" s="11" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A93" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="B93" s="12" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A94" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B94" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A95" s="7" t="s">
+        <v>75</v>
+      </c>
+      <c r="B95" s="12" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A96" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B96" s="12" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A97" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="B97" s="12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A98" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B98" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A99" s="8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B99" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A100" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="B100" s="12" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A101" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B101" s="12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A102" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B55" s="2" t="s">
+      <c r="B102" s="12" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A103" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B103" s="11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A104" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B104" s="11" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A105" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B105" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A106" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="B106" s="21" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>